<commit_message>
Applique les arbitrages validés du BMC v1.3 au dépôt
- Grille : 490 €/position de mise en service remplacent le dépôt de 900 € ;
  offre de lancement limitée au poste dédié ; clause de révision EUR/MGA ;
  12 mois fermes comme objectif de négociation ; autonomie visée vers deux mois.
- Moteur : coût complet agent de 3,5 M Ar, structure du lancement, équipement,
  réserves SLA et change, fondateur encadrant 5 positions, scénario 3 + 2.
- Pages de projection et de négociation, classeur Excel, générateur de devis,
  contrat et devis types, fiches d'offre, scripts et site alignés.
- Tests : nouvelles valeurs par défaut testées, anciens mécanismes sous LEGACY ;
  classeur vérifié cellule par cellule et formule par formule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VJeqYPw2rJL5Lhg99iejcR
</commit_message>
<xml_diff>
--- a/PROJECTION-FINANCES-SALVERYS.xlsx
+++ b/PROJECTION-FINANCES-SALVERYS.xlsx
@@ -879,7 +879,7 @@
       </c>
       <c r="B6" s="5">
         <f>MIN(Flux!L6:L29)</f>
-        <v>-4800.240000000001</v>
+        <v>-16948</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
       </c>
       <c r="B8" s="5">
         <f>MAX(0,-MIN(Flux!L6:L29))*1.3</f>
-        <v>6240.312000000001</v>
+        <v>22032.4</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
       </c>
       <c r="B9" s="5">
         <f>Flux!L29</f>
-        <v>24803.79999999998</v>
+        <v>50768</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
@@ -943,11 +943,11 @@
       </c>
       <c r="B10" s="5">
         <f>Contribution!E20</f>
-        <v>2339.7599999999998</v>
+        <v>3762</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Tous contrats actifs, hors onboarding, dépôt, impayés et taxes.</t>
+          <t>Tous contrats actifs, structure et réserves comprises, hors onboarding, équipement, impayés et taxes.</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="B11" s="8">
         <f>Flux!B29</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C11" s="6" t="inlineStr"/>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B12" s="8">
         <f>Flux!C29</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
@@ -987,11 +987,11 @@
       </c>
       <c r="B13" s="9">
         <f>Hypothèses!B14</f>
-        <v>843.0400000000001</v>
+        <v>730</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Salaire chargé, VoIP et coussin. Trois hypothèses non vérifiées le déterminent.</t>
+          <t>Coût complet agent tout compris + VoIP (arbitrage A7, à valider par la paie).</t>
         </is>
       </c>
     </row>
@@ -1003,11 +1003,11 @@
       </c>
       <c r="B14" s="9">
         <f>Grille!B13</f>
-        <v>944.2950000000001</v>
+        <v>856.9639175257732</v>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>En dessous, aucun volume ne rattrape le prix. Le plancher de PRICING.md est SOUS ce seuil.</t>
+          <t>En dessous, aucun volume ne rattrape le prix. Structure du lancement non comprise.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Impôts et TVA, comptabilité, assurance, frais bancaires et de change, équipement et liaisons de secours, recrutement au-delà du forfait d'onboarding, congés et remplacement, turnover, indemnités de rupture, dettes et créances existantes, dates réelles des factures annuelles. Le modèle A mutualisé (1 120 € / 400 tickets) et le télésecrétariat médical facturé à l'appel ne sont pas projetés : leur staffing n'est pas mesuré.</t>
+          <t>Impôts et TVA, assurance, amortissements comptables, recrutement au-delà du forfait d'onboarding, indemnités de rupture, dettes et créances existantes, dates réelles des factures annuelles. Le modèle A mutualisé (1 120 € / 400 tickets) et le télésecrétariat médical facturé à l'appel ne sont pas projetés : leur staffing n'est pas mesuré.</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1142,7 +1142,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Brut mensuel agent et manager</t>
+          <t>Brut mensuel manager (et agent si B39 = 0)</t>
         </is>
       </c>
       <c r="B6" s="13" t="n">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Décision direction 2026-08-14. À confirmer sur bulletins de paie.</t>
+          <t>Décision direction 2026-08-14. À confirmer sur bulletins de paie. Depuis le 2026-09-24, l'agent se chiffre au coût complet de la ligne 39.</t>
         </is>
       </c>
     </row>
@@ -1307,8 +1307,8 @@
         </is>
       </c>
       <c r="B14" s="19">
-        <f>((B6+MIN(B6,B10)*B8)/B7+B11)*(1+B13)</f>
-        <v>843.0400000000001</v>
+        <f>IF(B39&gt;0,B39/B7+B11,((B6+MIN(B6,B10)*B8)/B7+B11)*(1+B13))</f>
+        <v>730</v>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Calculé : (brut + cotisations plafonnées) ÷ change, plus VoIP, plus coussin.</t>
+          <t>Calculé : coût complet (ligne 39) ÷ change + VoIP, sans coussin. Si la ligne 39 vaut 0 : (brut + cotisations plafonnées) ÷ change, plus VoIP, plus coussin.</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
         </is>
       </c>
       <c r="B17" s="20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>0 = un manager dès la première position. Au-delà, doit correspondre à un temps réellement disponible.</t>
+          <t>Arbitrage A10 du 2026-09-24 : le fondateur encadre le lancement à 5 positions. Un manager s'ajoute à la 6e ; le forfait d'encadrement de la ligne 40 est alors à recalculer.</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
         </is>
       </c>
       <c r="B27" s="18" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>PRICING.md §3. AVANCE de trésorerie : intégralement rendue par crédit de facture.</t>
+          <t>SUPPRIMÉ de la grille le 2026-09-24 (arbitrage A1), remplacé par les frais de mise en service. Gardé pour simuler l'ancien dépôt rendu par crédit de facture.</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="B28" s="18" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
@@ -1580,7 +1580,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>PRICING.md §3.</t>
+          <t>Ancien mécanisme, à 0.</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>PRICING.md §3.</t>
+          <t>Ancien mécanisme.</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1628,7 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Frais d'activation par contrat</t>
+          <t>Frais de mise en service par contrat</t>
         </is>
       </c>
       <c r="B31" s="18" t="n">
@@ -1641,18 +1641,18 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>JAMAIS rendus, contrairement au dépôt. PRICING.md §3 dit qu'il n'y en a pas : les activer MODIFIE LA GRILLE.</t>
+          <t>Part fixe éventuelle. PRICING.md §3 n'en prévoit pas.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Frais d'activation par position</t>
+          <t>Frais de mise en service par position</t>
         </is>
       </c>
       <c r="B32" s="18" t="n">
-        <v>0</v>
+        <v>490</v>
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Idem. Une avance rendue se défend par « vous ne le payez pas » ; un frais acquis, non.</t>
+          <t>PRICING.md §3, arbitrage A1 du 2026-09-24 : 490 €/position à la signature, acquis, non imputés sur les mensualités.</t>
         </is>
       </c>
     </row>
@@ -1688,11 +1688,11 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Taxes et frais sur CA encaissé</t>
+          <t>Banque, change et taxes sur CA encaissé</t>
         </is>
       </c>
       <c r="B34" s="16" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Impôt, TVA, frais bancaires. Non renseigné faute de taux vérifiés.</t>
+          <t>Arbitrage A9 : 1 % de frais bancaires et risque de change. Taxes non comprises : taux non vérifiés.</t>
         </is>
       </c>
     </row>
@@ -1736,8 +1736,119 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="12" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>ARBITRAGES DU 2026-09-24 (BMC v1.3)</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="n"/>
+      <c r="C38" s="11" t="n"/>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="11" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Coût complet agent, tout compris</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>Ar / mois</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Arbitrage A7 : rémunération, charges, congés, absences, formation et remplacement. À VALIDER PAR LA PAIE : le brut de la ligne 6 chargé n'y tient pas. 0 = calcul par le brut.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Structure dès la 1re embauche</t>
+        </is>
+      </c>
+      <c r="B40" s="18" t="n">
+        <v>2220</v>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>€ / mois</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>Arbitrage A8, hypothèse pessimiste : encadrement / QA 600 + loyer 60 m² 720 + double fibre 300 + RH / paie / comptable 300 + énergie 300. Payée tant qu'un agent est en poste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Poste de travail par position</t>
+        </is>
+      </c>
+      <c r="B41" s="18" t="n">
+        <v>800</v>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Laptop + écran, 4 M Ar, décaissés à la signature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Groupe électrogène + UPS</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="n">
+        <v>450</v>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>2,25 M Ar, décaissés une fois, au premier mois avec du personnel. À tester avant d'être promis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Provision avoirs SLA sur CA encaissé</t>
+        </is>
+      </c>
+      <c r="B43" s="16" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Arbitrage A9 : avoir de 20 % au plus un mois sur douze = 1,7 % du CA ; provision de 2 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="12" t="inlineStr">
         <is>
           <t>Aucun chiffre de ce classeur ne représente une dépense constatée tant que les factures, la paie et le solde bancaire n'ont pas été rapprochés. Trois hypothèses pèsent sur tout le reste : le taux de cotisation, le plafond et le taux de change. Elles fixent le coût d'une position, donc toute marge annoncée.</t>
         </is>
@@ -1745,7 +1856,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A45:D45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1884,7 +1995,7 @@
       </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>À RÉVISER : n'est rentable à aucun volume. Chaque tranche de 8 positions à ce prix creuse le résultat d'environ 194 €/mois.</t>
+          <t>À RÉVISER. Garde-fou de négociation, pas seuil de rentabilité : comparer à la ligne 13, puis chiffrer le contrat avec la structure du lancement.</t>
         </is>
       </c>
     </row>
@@ -1895,12 +2006,12 @@
         </is>
       </c>
       <c r="B13" s="23">
-        <f>Hypothèses!B14+Hypothèses!B15/Hypothèses!B16</f>
-        <v>944.2950000000001</v>
+        <f>(Hypothèses!B14+Hypothèses!B15/Hypothèses!B16)/(1-Hypothèses!B34-Hypothèses!B43)</f>
+        <v>856.9639175257732</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Coût d'un agent plus sa quote-part de manager. En dessous, aucun volume ne rattrape le prix.</t>
+          <t>Coût d'un agent plus sa quote-part de manager, réserves sur CA comprises. En dessous, aucun volume ne rattrape le prix. Structure du lancement non comprise.</t>
         </is>
       </c>
     </row>
@@ -1964,7 +2075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1978,6 +2089,7 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -2042,19 +2154,24 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Frais d'activation</t>
+          <t>Mise en service</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Crédit de dépôt / facture</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Postes de travail</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>Contrat 1</t>
+          <t>Client A</t>
         </is>
       </c>
       <c r="B6" s="20" t="n">
@@ -2066,7 +2183,7 @@
         </is>
       </c>
       <c r="D6" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" s="27" t="inlineStr">
         <is>
@@ -2076,37 +2193,41 @@
       <c r="F6" s="18" t="n"/>
       <c r="G6" s="28">
         <f>IF($D6="",0,IF($E6="mb",MIN($D6,Grille!$B$5)*INDEX(Grille!$B$8:$B$9,MATCH($C6,Grille!$A$8:$A$9,0))+MAX(0,$D6-Grille!$B$5)*INDEX(Grille!$C$8:$C$9,MATCH($C6,Grille!$A$8:$A$9,0)),$D6*$F6))</f>
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="H6" s="29">
         <f>IF($D6="",0,Hypothèses!$B$21+$D6*Hypothèses!$B$22)</f>
-        <v>1200</v>
+        <v>1600</v>
       </c>
       <c r="I6" s="29">
         <f>IF($D6="",0,$D6*Hypothèses!$B$27)</f>
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="J6" s="29">
         <f>IF($D6="",0,Hypothèses!$B$31+$D6*Hypothèses!$B$32)</f>
-        <v>0</v>
+        <v>1470</v>
       </c>
       <c r="K6" s="29">
         <f>IF($D6="",0,$D6*Hypothèses!$B$28)</f>
-        <v>600</v>
+        <v>0</v>
+      </c>
+      <c r="L6" s="29">
+        <f>IF($D6="",0,$D6*Hypothèses!$B$41)</f>
+        <v>2400</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>Contrat 2</t>
+          <t>Client B</t>
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>support</t>
+          <t>helpdesk</t>
         </is>
       </c>
       <c r="D7" s="20" t="n">
@@ -2120,7 +2241,7 @@
       <c r="F7" s="18" t="n"/>
       <c r="G7" s="28">
         <f>IF($D7="",0,IF($E7="mb",MIN($D7,Grille!$B$5)*INDEX(Grille!$B$8:$B$9,MATCH($C7,Grille!$A$8:$A$9,0))+MAX(0,$D7-Grille!$B$5)*INDEX(Grille!$C$8:$C$9,MATCH($C7,Grille!$A$8:$A$9,0)),$D7*$F7))</f>
-        <v>3400</v>
+        <v>4000</v>
       </c>
       <c r="H7" s="29">
         <f>IF($D7="",0,Hypothèses!$B$21+$D7*Hypothèses!$B$22)</f>
@@ -2128,15 +2249,19 @@
       </c>
       <c r="I7" s="29">
         <f>IF($D7="",0,$D7*Hypothèses!$B$27)</f>
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="J7" s="29">
         <f>IF($D7="",0,Hypothèses!$B$31+$D7*Hypothèses!$B$32)</f>
-        <v>0</v>
+        <v>980</v>
       </c>
       <c r="K7" s="29">
         <f>IF($D7="",0,$D7*Hypothèses!$B$28)</f>
-        <v>600</v>
+        <v>0</v>
+      </c>
+      <c r="L7" s="29">
+        <f>IF($D7="",0,$D7*Hypothèses!$B$41)</f>
+        <v>1600</v>
       </c>
     </row>
     <row r="8">
@@ -2166,6 +2291,10 @@
         <f>IF($D8="",0,$D8*Hypothèses!$B$28)</f>
         <v>0</v>
       </c>
+      <c r="L8" s="29">
+        <f>IF($D8="",0,$D8*Hypothèses!$B$41)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="26" t="inlineStr"/>
@@ -2194,6 +2323,10 @@
         <f>IF($D9="",0,$D9*Hypothèses!$B$28)</f>
         <v>0</v>
       </c>
+      <c r="L9" s="29">
+        <f>IF($D9="",0,$D9*Hypothèses!$B$41)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="26" t="inlineStr"/>
@@ -2222,6 +2355,10 @@
         <f>IF($D10="",0,$D10*Hypothèses!$B$28)</f>
         <v>0</v>
       </c>
+      <c r="L10" s="29">
+        <f>IF($D10="",0,$D10*Hypothèses!$B$41)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="26" t="inlineStr"/>
@@ -2250,6 +2387,10 @@
         <f>IF($D11="",0,$D11*Hypothèses!$B$28)</f>
         <v>0</v>
       </c>
+      <c r="L11" s="29">
+        <f>IF($D11="",0,$D11*Hypothèses!$B$41)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="26" t="inlineStr"/>
@@ -2278,6 +2419,10 @@
         <f>IF($D12="",0,$D12*Hypothèses!$B$28)</f>
         <v>0</v>
       </c>
+      <c r="L12" s="29">
+        <f>IF($D12="",0,$D12*Hypothèses!$B$41)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="26" t="inlineStr"/>
@@ -2306,6 +2451,10 @@
         <f>IF($D13="",0,$D13*Hypothèses!$B$28)</f>
         <v>0</v>
       </c>
+      <c r="L13" s="29">
+        <f>IF($D13="",0,$D13*Hypothèses!$B$41)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
@@ -2316,7 +2465,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="A15:L15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2406,12 +2555,12 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Onboarding et équipement</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Structure et réserves</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -2468,11 +2617,11 @@
         <v>0</v>
       </c>
       <c r="I6" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A6)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A6)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A6)*Contrats!$L$6:$L$13)-IF(AND($B6&gt;0,COUNTIF($B$6:$B6,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J6" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G6*Hypothèses!$B$34)</f>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B6&gt;0,Hypothèses!$B$40,0)+$G6*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
         <v>-68</v>
       </c>
       <c r="K6" s="29">
@@ -2525,11 +2674,11 @@
         <v>0</v>
       </c>
       <c r="I7" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A7)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A7)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A7)*Contrats!$L$6:$L$13)-IF(AND($B7&gt;0,COUNTIF($B$6:$B7,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J7" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G7*Hypothèses!$B$34)</f>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B7&gt;0,Hypothèses!$B$40,0)+$G7*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
         <v>-68</v>
       </c>
       <c r="K7" s="34">
@@ -2582,11 +2731,11 @@
         <v>0</v>
       </c>
       <c r="I8" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A8)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A8)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A8)*Contrats!$L$6:$L$13)-IF(AND($B8&gt;0,COUNTIF($B$6:$B8,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J8" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G8*Hypothèses!$B$34)</f>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B8&gt;0,Hypothèses!$B$40,0)+$G8*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
         <v>-68</v>
       </c>
       <c r="K8" s="29">
@@ -2620,11 +2769,11 @@
       </c>
       <c r="D9" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A9)*Contrats!$I$6:$I$13)</f>
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="E9" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A9)*Contrats!$J$6:$J$13)</f>
-        <v>0</v>
+        <v>2450</v>
       </c>
       <c r="F9" s="34">
         <f>SUMPRODUCT(($A9&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A9-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A9-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
@@ -2639,20 +2788,20 @@
         <v>0</v>
       </c>
       <c r="I9" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A9)*Contrats!$H$6:$H$13)</f>
-        <v>-1200</v>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A9)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A9)*Contrats!$L$6:$L$13)-IF(AND($B9&gt;0,COUNTIF($B$6:$B9,"&gt;0")=1),Hypothèses!$B$42,0)</f>
+        <v>-6800</v>
       </c>
       <c r="J9" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G9*Hypothèses!$B$34)</f>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B9&gt;0,Hypothèses!$B$40,0)+$G9*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
         <v>-68</v>
       </c>
       <c r="K9" s="34">
         <f>$G9+$E9+$H9+$I9+$J9</f>
-        <v>-1268</v>
+        <v>-4418</v>
       </c>
       <c r="L9" s="35">
         <f>L8+$D9+$K9</f>
-        <v>328</v>
+        <v>-4622</v>
       </c>
       <c r="M9" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A9&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
@@ -2669,11 +2818,11 @@
       </c>
       <c r="B10" s="31">
         <f>$M10+$N10</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C10" s="31">
         <f>IF($B10&lt;=Hypothèses!$B$17,0,IF($M10=0,0,CEILING($M10/Hypothèses!$B$16,1))+IF($N10=0,0,CEILING($N10/Hypothèses!$B$16,1)))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10" s="29">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A10)*Contrats!$I$6:$I$13)</f>
@@ -2693,27 +2842,27 @@
       </c>
       <c r="H10" s="29">
         <f>-($B10*Hypothèses!$B$14+$C10*Hypothèses!$B$15)</f>
-        <v>-2496.1200000000003</v>
+        <v>-3650</v>
       </c>
       <c r="I10" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A10)*Contrats!$H$6:$H$13)</f>
-        <v>0</v>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A10)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A10)*Contrats!$L$6:$L$13)-IF(AND($B10&gt;0,COUNTIF($B$6:$B10,"&gt;0")=1),Hypothèses!$B$42,0)</f>
+        <v>-450</v>
       </c>
       <c r="J10" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G10*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B10&gt;0,Hypothèses!$B$40,0)+$G10*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2288</v>
       </c>
       <c r="K10" s="29">
         <f>$G10+$E10+$H10+$I10+$J10</f>
-        <v>-2564.1200000000003</v>
+        <v>-6388</v>
       </c>
       <c r="L10" s="28">
         <f>L9+$D10+$K10</f>
-        <v>-2236.1200000000003</v>
+        <v>-11010</v>
       </c>
       <c r="M10" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A10&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N10" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A10&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
@@ -2726,11 +2875,11 @@
       </c>
       <c r="B11" s="33">
         <f>$M11+$N11</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C11" s="33">
         <f>IF($B11&lt;=Hypothèses!$B$17,0,IF($M11=0,0,CEILING($M11/Hypothèses!$B$16,1))+IF($N11=0,0,CEILING($N11/Hypothèses!$B$16,1)))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A11)*Contrats!$I$6:$I$13)</f>
@@ -2742,7 +2891,7 @@
       </c>
       <c r="F11" s="34">
         <f>SUMPRODUCT(($A11&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A11-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A11-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>3400</v>
+        <v>10000</v>
       </c>
       <c r="G11" s="34">
         <f>(SUMPRODUCT(($A11&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A11-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A11-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
@@ -2750,27 +2899,27 @@
       </c>
       <c r="H11" s="34">
         <f>-($B11*Hypothèses!$B$14+$C11*Hypothèses!$B$15)</f>
-        <v>-2496.1200000000003</v>
+        <v>-3650</v>
       </c>
       <c r="I11" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A11)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A11)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A11)*Contrats!$L$6:$L$13)-IF(AND($B11&gt;0,COUNTIF($B$6:$B11,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J11" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G11*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B11&gt;0,Hypothèses!$B$40,0)+$G11*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2288</v>
       </c>
       <c r="K11" s="34">
         <f>$G11+$E11+$H11+$I11+$J11</f>
-        <v>-2564.1200000000003</v>
+        <v>-5938</v>
       </c>
       <c r="L11" s="35">
         <f>L10+$D11+$K11</f>
-        <v>-4800.240000000001</v>
+        <v>-16948</v>
       </c>
       <c r="M11" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A11&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N11" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A11&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
@@ -2783,11 +2932,11 @@
       </c>
       <c r="B12" s="31">
         <f>$M12+$N12</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C12" s="31">
         <f>IF($B12&lt;=Hypothèses!$B$17,0,IF($M12=0,0,CEILING($M12/Hypothèses!$B$16,1))+IF($N12=0,0,CEILING($N12/Hypothèses!$B$16,1)))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="29">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A12)*Contrats!$I$6:$I$13)</f>
@@ -2799,35 +2948,35 @@
       </c>
       <c r="F12" s="29">
         <f>SUMPRODUCT(($A12&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A12-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A12-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>3400</v>
+        <v>10000</v>
       </c>
       <c r="G12" s="29">
         <f>(SUMPRODUCT(($A12&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A12-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A12-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>3400</v>
+        <v>10000</v>
       </c>
       <c r="H12" s="29">
         <f>-($B12*Hypothèses!$B$14+$C12*Hypothèses!$B$15)</f>
-        <v>-2496.1200000000003</v>
+        <v>-3650</v>
       </c>
       <c r="I12" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A12)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A12)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A12)*Contrats!$L$6:$L$13)-IF(AND($B12&gt;0,COUNTIF($B$6:$B12,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J12" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G12*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B12&gt;0,Hypothèses!$B$40,0)+$G12*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K12" s="29">
         <f>$G12+$E12+$H12+$I12+$J12</f>
-        <v>835.8799999999997</v>
+        <v>3762</v>
       </c>
       <c r="L12" s="28">
         <f>L11+$D12+$K12</f>
-        <v>-3964.360000000001</v>
+        <v>-13186</v>
       </c>
       <c r="M12" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A12&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N12" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A12&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
@@ -2840,11 +2989,11 @@
       </c>
       <c r="B13" s="33">
         <f>$M13+$N13</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C13" s="33">
         <f>IF($B13&lt;=Hypothèses!$B$17,0,IF($M13=0,0,CEILING($M13/Hypothèses!$B$16,1))+IF($N13=0,0,CEILING($N13/Hypothèses!$B$16,1)))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A13)*Contrats!$I$6:$I$13)</f>
@@ -2856,35 +3005,35 @@
       </c>
       <c r="F13" s="34">
         <f>SUMPRODUCT(($A13&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A13-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A13-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>3400</v>
+        <v>10000</v>
       </c>
       <c r="G13" s="34">
         <f>(SUMPRODUCT(($A13&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A13-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A13-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>3400</v>
+        <v>10000</v>
       </c>
       <c r="H13" s="34">
         <f>-($B13*Hypothèses!$B$14+$C13*Hypothèses!$B$15)</f>
-        <v>-2496.1200000000003</v>
+        <v>-3650</v>
       </c>
       <c r="I13" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A13)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A13)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A13)*Contrats!$L$6:$L$13)-IF(AND($B13&gt;0,COUNTIF($B$6:$B13,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J13" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G13*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B13&gt;0,Hypothèses!$B$40,0)+$G13*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K13" s="34">
         <f>$G13+$E13+$H13+$I13+$J13</f>
-        <v>835.8799999999997</v>
+        <v>3762</v>
       </c>
       <c r="L13" s="35">
         <f>L12+$D13+$K13</f>
-        <v>-3128.4800000000014</v>
+        <v>-9424</v>
       </c>
       <c r="M13" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A13&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N13" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A13&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
@@ -2897,15 +3046,15 @@
       </c>
       <c r="B14" s="31">
         <f>$M14+$N14</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C14" s="31">
         <f>IF($B14&lt;=Hypothèses!$B$17,0,IF($M14=0,0,CEILING($M14/Hypothèses!$B$16,1))+IF($N14=0,0,CEILING($N14/Hypothèses!$B$16,1)))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" s="29">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A14)*Contrats!$I$6:$I$13)</f>
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="E14" s="29">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A14)*Contrats!$J$6:$J$13)</f>
@@ -2913,35 +3062,35 @@
       </c>
       <c r="F14" s="29">
         <f>SUMPRODUCT(($A14&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A14-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A14-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="G14" s="29">
         <f>(SUMPRODUCT(($A14&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A14-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A14-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>3400</v>
+        <v>10000</v>
       </c>
       <c r="H14" s="29">
         <f>-($B14*Hypothèses!$B$14+$C14*Hypothèses!$B$15)</f>
-        <v>-2496.1200000000003</v>
+        <v>-3650</v>
       </c>
       <c r="I14" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A14)*Contrats!$H$6:$H$13)</f>
-        <v>-1200</v>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A14)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A14)*Contrats!$L$6:$L$13)-IF(AND($B14&gt;0,COUNTIF($B$6:$B14,"&gt;0")=1),Hypothèses!$B$42,0)</f>
+        <v>0</v>
       </c>
       <c r="J14" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G14*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B14&gt;0,Hypothèses!$B$40,0)+$G14*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K14" s="29">
         <f>$G14+$E14+$H14+$I14+$J14</f>
-        <v>-364.12000000000035</v>
+        <v>3762</v>
       </c>
       <c r="L14" s="28">
         <f>L13+$D14+$K14</f>
-        <v>-1692.6000000000017</v>
+        <v>-5662</v>
       </c>
       <c r="M14" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A14&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N14" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A14&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
@@ -2954,11 +3103,11 @@
       </c>
       <c r="B15" s="33">
         <f>$M15+$N15</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15" s="33">
         <f>IF($B15&lt;=Hypothèses!$B$17,0,IF($M15=0,0,CEILING($M15/Hypothèses!$B$16,1))+IF($N15=0,0,CEILING($N15/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D15" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A15)*Contrats!$I$6:$I$13)</f>
@@ -2970,39 +3119,39 @@
       </c>
       <c r="F15" s="34">
         <f>SUMPRODUCT(($A15&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A15-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A15-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="G15" s="34">
         <f>(SUMPRODUCT(($A15&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A15-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A15-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="H15" s="34">
         <f>-($B15*Hypothèses!$B$14+$C15*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I15" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A15)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A15)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A15)*Contrats!$L$6:$L$13)-IF(AND($B15&gt;0,COUNTIF($B$6:$B15,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J15" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G15*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B15&gt;0,Hypothèses!$B$40,0)+$G15*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K15" s="34">
         <f>$G15+$E15+$H15+$I15+$J15</f>
-        <v>-1060.2400000000007</v>
+        <v>3762</v>
       </c>
       <c r="L15" s="35">
         <f>L14+$D15+$K15</f>
-        <v>-2752.8400000000024</v>
+        <v>-1900</v>
       </c>
       <c r="M15" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A15&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N15" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A15&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -3011,11 +3160,11 @@
       </c>
       <c r="B16" s="31">
         <f>$M16+$N16</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C16" s="31">
         <f>IF($B16&lt;=Hypothèses!$B$17,0,IF($M16=0,0,CEILING($M16/Hypothèses!$B$16,1))+IF($N16=0,0,CEILING($N16/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D16" s="29">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A16)*Contrats!$I$6:$I$13)</f>
@@ -3027,39 +3176,39 @@
       </c>
       <c r="F16" s="29">
         <f>SUMPRODUCT(($A16&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A16-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A16-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>6800</v>
+        <v>10000</v>
       </c>
       <c r="G16" s="29">
         <f>(SUMPRODUCT(($A16&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A16-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A16-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="H16" s="29">
         <f>-($B16*Hypothèses!$B$14+$C16*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I16" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A16)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A16)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A16)*Contrats!$L$6:$L$13)-IF(AND($B16&gt;0,COUNTIF($B$6:$B16,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J16" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G16*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B16&gt;0,Hypothèses!$B$40,0)+$G16*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K16" s="29">
         <f>$G16+$E16+$H16+$I16+$J16</f>
-        <v>-1060.2400000000007</v>
+        <v>3762</v>
       </c>
       <c r="L16" s="28">
         <f>L15+$D16+$K16</f>
-        <v>-3813.080000000003</v>
+        <v>1862</v>
       </c>
       <c r="M16" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A16&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N16" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A16&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -3068,11 +3217,11 @@
       </c>
       <c r="B17" s="33">
         <f>$M17+$N17</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C17" s="33">
         <f>IF($B17&lt;=Hypothèses!$B$17,0,IF($M17=0,0,CEILING($M17/Hypothèses!$B$16,1))+IF($N17=0,0,CEILING($N17/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D17" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A17)*Contrats!$I$6:$I$13)</f>
@@ -3084,39 +3233,39 @@
       </c>
       <c r="F17" s="34">
         <f>SUMPRODUCT(($A17&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A17-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A17-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>6800</v>
+        <v>10000</v>
       </c>
       <c r="G17" s="34">
         <f>(SUMPRODUCT(($A17&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A17-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A17-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>6800</v>
+        <v>10000</v>
       </c>
       <c r="H17" s="34">
         <f>-($B17*Hypothèses!$B$14+$C17*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I17" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A17)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A17)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A17)*Contrats!$L$6:$L$13)-IF(AND($B17&gt;0,COUNTIF($B$6:$B17,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J17" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G17*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B17&gt;0,Hypothèses!$B$40,0)+$G17*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K17" s="34">
         <f>$G17+$E17+$H17+$I17+$J17</f>
-        <v>1739.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L17" s="35">
         <f>L16+$D17+$K17</f>
-        <v>-2073.320000000004</v>
+        <v>5624</v>
       </c>
       <c r="M17" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A17&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N17" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A17&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -3125,11 +3274,11 @@
       </c>
       <c r="B18" s="31">
         <f>$M18+$N18</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C18" s="31">
         <f>IF($B18&lt;=Hypothèses!$B$17,0,IF($M18=0,0,CEILING($M18/Hypothèses!$B$16,1))+IF($N18=0,0,CEILING($N18/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D18" s="29">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A18)*Contrats!$I$6:$I$13)</f>
@@ -3141,39 +3290,39 @@
       </c>
       <c r="F18" s="29">
         <f>SUMPRODUCT(($A18&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A18-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A18-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>6800</v>
+        <v>10000</v>
       </c>
       <c r="G18" s="29">
         <f>(SUMPRODUCT(($A18&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A18-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A18-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>6800</v>
+        <v>10000</v>
       </c>
       <c r="H18" s="29">
         <f>-($B18*Hypothèses!$B$14+$C18*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I18" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A18)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A18)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A18)*Contrats!$L$6:$L$13)-IF(AND($B18&gt;0,COUNTIF($B$6:$B18,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J18" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G18*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B18&gt;0,Hypothèses!$B$40,0)+$G18*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K18" s="29">
         <f>$G18+$E18+$H18+$I18+$J18</f>
-        <v>1739.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L18" s="28">
         <f>L17+$D18+$K18</f>
-        <v>-333.5600000000045</v>
+        <v>9386</v>
       </c>
       <c r="M18" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A18&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N18" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A18&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -3182,11 +3331,11 @@
       </c>
       <c r="B19" s="33">
         <f>$M19+$N19</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" s="33">
         <f>IF($B19&lt;=Hypothèses!$B$17,0,IF($M19=0,0,CEILING($M19/Hypothèses!$B$16,1))+IF($N19=0,0,CEILING($N19/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D19" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A19)*Contrats!$I$6:$I$13)</f>
@@ -3198,39 +3347,39 @@
       </c>
       <c r="F19" s="34">
         <f>SUMPRODUCT(($A19&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A19-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A19-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="G19" s="34">
         <f>(SUMPRODUCT(($A19&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A19-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A19-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>6800</v>
+        <v>10000</v>
       </c>
       <c r="H19" s="34">
         <f>-($B19*Hypothèses!$B$14+$C19*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I19" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A19)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A19)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A19)*Contrats!$L$6:$L$13)-IF(AND($B19&gt;0,COUNTIF($B$6:$B19,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J19" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G19*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B19&gt;0,Hypothèses!$B$40,0)+$G19*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K19" s="34">
         <f>$G19+$E19+$H19+$I19+$J19</f>
-        <v>1739.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L19" s="35">
         <f>L18+$D19+$K19</f>
-        <v>1406.1999999999948</v>
+        <v>13148</v>
       </c>
       <c r="M19" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A19&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N19" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A19&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -3239,11 +3388,11 @@
       </c>
       <c r="B20" s="31">
         <f>$M20+$N20</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C20" s="31">
         <f>IF($B20&lt;=Hypothèses!$B$17,0,IF($M20=0,0,CEILING($M20/Hypothèses!$B$16,1))+IF($N20=0,0,CEILING($N20/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D20" s="29">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A20)*Contrats!$I$6:$I$13)</f>
@@ -3255,39 +3404,39 @@
       </c>
       <c r="F20" s="29">
         <f>SUMPRODUCT(($A20&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A20-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A20-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="G20" s="29">
         <f>(SUMPRODUCT(($A20&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A20-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A20-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="H20" s="29">
         <f>-($B20*Hypothèses!$B$14+$C20*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I20" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A20)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A20)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A20)*Contrats!$L$6:$L$13)-IF(AND($B20&gt;0,COUNTIF($B$6:$B20,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J20" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G20*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B20&gt;0,Hypothèses!$B$40,0)+$G20*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K20" s="29">
         <f>$G20+$E20+$H20+$I20+$J20</f>
-        <v>2339.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L20" s="28">
         <f>L19+$D20+$K20</f>
-        <v>3745.959999999994</v>
+        <v>16910</v>
       </c>
       <c r="M20" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A20&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N20" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A20&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -3296,11 +3445,11 @@
       </c>
       <c r="B21" s="33">
         <f>$M21+$N21</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21" s="33">
         <f>IF($B21&lt;=Hypothèses!$B$17,0,IF($M21=0,0,CEILING($M21/Hypothèses!$B$16,1))+IF($N21=0,0,CEILING($N21/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D21" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A21)*Contrats!$I$6:$I$13)</f>
@@ -3312,39 +3461,39 @@
       </c>
       <c r="F21" s="34">
         <f>SUMPRODUCT(($A21&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A21-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A21-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="G21" s="34">
         <f>(SUMPRODUCT(($A21&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A21-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A21-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="H21" s="34">
         <f>-($B21*Hypothèses!$B$14+$C21*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I21" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A21)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A21)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A21)*Contrats!$L$6:$L$13)-IF(AND($B21&gt;0,COUNTIF($B$6:$B21,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J21" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G21*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B21&gt;0,Hypothèses!$B$40,0)+$G21*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K21" s="34">
         <f>$G21+$E21+$H21+$I21+$J21</f>
-        <v>2339.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L21" s="35">
         <f>L20+$D21+$K21</f>
-        <v>6085.719999999994</v>
+        <v>20672</v>
       </c>
       <c r="M21" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A21&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N21" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A21&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -3353,11 +3502,11 @@
       </c>
       <c r="B22" s="31">
         <f>$M22+$N22</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22" s="31">
         <f>IF($B22&lt;=Hypothèses!$B$17,0,IF($M22=0,0,CEILING($M22/Hypothèses!$B$16,1))+IF($N22=0,0,CEILING($N22/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D22" s="29">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A22)*Contrats!$I$6:$I$13)</f>
@@ -3369,39 +3518,39 @@
       </c>
       <c r="F22" s="29">
         <f>SUMPRODUCT(($A22&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A22-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A22-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="G22" s="29">
         <f>(SUMPRODUCT(($A22&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A22-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A22-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="H22" s="29">
         <f>-($B22*Hypothèses!$B$14+$C22*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I22" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A22)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A22)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A22)*Contrats!$L$6:$L$13)-IF(AND($B22&gt;0,COUNTIF($B$6:$B22,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J22" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G22*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B22&gt;0,Hypothèses!$B$40,0)+$G22*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K22" s="29">
         <f>$G22+$E22+$H22+$I22+$J22</f>
-        <v>2339.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L22" s="28">
         <f>L21+$D22+$K22</f>
-        <v>8425.479999999992</v>
+        <v>24434</v>
       </c>
       <c r="M22" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A22&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N22" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A22&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -3410,11 +3559,11 @@
       </c>
       <c r="B23" s="33">
         <f>$M23+$N23</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C23" s="33">
         <f>IF($B23&lt;=Hypothèses!$B$17,0,IF($M23=0,0,CEILING($M23/Hypothèses!$B$16,1))+IF($N23=0,0,CEILING($N23/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D23" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A23)*Contrats!$I$6:$I$13)</f>
@@ -3426,39 +3575,39 @@
       </c>
       <c r="F23" s="34">
         <f>SUMPRODUCT(($A23&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A23-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A23-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="G23" s="34">
         <f>(SUMPRODUCT(($A23&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A23-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A23-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="H23" s="34">
         <f>-($B23*Hypothèses!$B$14+$C23*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I23" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A23)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A23)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A23)*Contrats!$L$6:$L$13)-IF(AND($B23&gt;0,COUNTIF($B$6:$B23,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J23" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G23*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B23&gt;0,Hypothèses!$B$40,0)+$G23*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K23" s="34">
         <f>$G23+$E23+$H23+$I23+$J23</f>
-        <v>2339.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L23" s="35">
         <f>L22+$D23+$K23</f>
-        <v>10765.23999999999</v>
+        <v>28196</v>
       </c>
       <c r="M23" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A23&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N23" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A23&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -3467,11 +3616,11 @@
       </c>
       <c r="B24" s="31">
         <f>$M24+$N24</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C24" s="31">
         <f>IF($B24&lt;=Hypothèses!$B$17,0,IF($M24=0,0,CEILING($M24/Hypothèses!$B$16,1))+IF($N24=0,0,CEILING($N24/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D24" s="29">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A24)*Contrats!$I$6:$I$13)</f>
@@ -3483,39 +3632,39 @@
       </c>
       <c r="F24" s="29">
         <f>SUMPRODUCT(($A24&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A24-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A24-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="G24" s="29">
         <f>(SUMPRODUCT(($A24&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A24-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A24-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="H24" s="29">
         <f>-($B24*Hypothèses!$B$14+$C24*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I24" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A24)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A24)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A24)*Contrats!$L$6:$L$13)-IF(AND($B24&gt;0,COUNTIF($B$6:$B24,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J24" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G24*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B24&gt;0,Hypothèses!$B$40,0)+$G24*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K24" s="29">
         <f>$G24+$E24+$H24+$I24+$J24</f>
-        <v>2339.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L24" s="28">
         <f>L23+$D24+$K24</f>
-        <v>13104.999999999989</v>
+        <v>31958</v>
       </c>
       <c r="M24" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A24&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N24" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A24&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -3524,11 +3673,11 @@
       </c>
       <c r="B25" s="33">
         <f>$M25+$N25</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25" s="33">
         <f>IF($B25&lt;=Hypothèses!$B$17,0,IF($M25=0,0,CEILING($M25/Hypothèses!$B$16,1))+IF($N25=0,0,CEILING($N25/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D25" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A25)*Contrats!$I$6:$I$13)</f>
@@ -3540,39 +3689,39 @@
       </c>
       <c r="F25" s="34">
         <f>SUMPRODUCT(($A25&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A25-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A25-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="G25" s="34">
         <f>(SUMPRODUCT(($A25&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A25-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A25-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="H25" s="34">
         <f>-($B25*Hypothèses!$B$14+$C25*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I25" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A25)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A25)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A25)*Contrats!$L$6:$L$13)-IF(AND($B25&gt;0,COUNTIF($B$6:$B25,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J25" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G25*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B25&gt;0,Hypothèses!$B$40,0)+$G25*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K25" s="34">
         <f>$G25+$E25+$H25+$I25+$J25</f>
-        <v>2339.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L25" s="35">
         <f>L24+$D25+$K25</f>
-        <v>15444.759999999987</v>
+        <v>35720</v>
       </c>
       <c r="M25" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A25&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N25" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A25&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -3581,11 +3730,11 @@
       </c>
       <c r="B26" s="31">
         <f>$M26+$N26</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C26" s="31">
         <f>IF($B26&lt;=Hypothèses!$B$17,0,IF($M26=0,0,CEILING($M26/Hypothèses!$B$16,1))+IF($N26=0,0,CEILING($N26/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D26" s="29">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A26)*Contrats!$I$6:$I$13)</f>
@@ -3597,39 +3746,39 @@
       </c>
       <c r="F26" s="29">
         <f>SUMPRODUCT(($A26&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="G26" s="29">
         <f>(SUMPRODUCT(($A26&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A26-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A26-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="H26" s="29">
         <f>-($B26*Hypothèses!$B$14+$C26*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I26" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A26)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A26)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A26)*Contrats!$L$6:$L$13)-IF(AND($B26&gt;0,COUNTIF($B$6:$B26,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J26" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G26*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B26&gt;0,Hypothèses!$B$40,0)+$G26*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K26" s="29">
         <f>$G26+$E26+$H26+$I26+$J26</f>
-        <v>2339.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L26" s="28">
         <f>L25+$D26+$K26</f>
-        <v>17784.519999999986</v>
+        <v>39482</v>
       </c>
       <c r="M26" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A26&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N26" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A26&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -3638,11 +3787,11 @@
       </c>
       <c r="B27" s="33">
         <f>$M27+$N27</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C27" s="33">
         <f>IF($B27&lt;=Hypothèses!$B$17,0,IF($M27=0,0,CEILING($M27/Hypothèses!$B$16,1))+IF($N27=0,0,CEILING($N27/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D27" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A27)*Contrats!$I$6:$I$13)</f>
@@ -3654,39 +3803,39 @@
       </c>
       <c r="F27" s="34">
         <f>SUMPRODUCT(($A27&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A27-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A27-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="G27" s="34">
         <f>(SUMPRODUCT(($A27&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A27-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A27-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="H27" s="34">
         <f>-($B27*Hypothèses!$B$14+$C27*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I27" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A27)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A27)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A27)*Contrats!$L$6:$L$13)-IF(AND($B27&gt;0,COUNTIF($B$6:$B27,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J27" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G27*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B27&gt;0,Hypothèses!$B$40,0)+$G27*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K27" s="34">
         <f>$G27+$E27+$H27+$I27+$J27</f>
-        <v>2339.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L27" s="35">
         <f>L26+$D27+$K27</f>
-        <v>20124.279999999984</v>
+        <v>43244</v>
       </c>
       <c r="M27" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A27&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N27" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A27&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -3695,11 +3844,11 @@
       </c>
       <c r="B28" s="31">
         <f>$M28+$N28</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C28" s="31">
         <f>IF($B28&lt;=Hypothèses!$B$17,0,IF($M28=0,0,CEILING($M28/Hypothèses!$B$16,1))+IF($N28=0,0,CEILING($N28/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D28" s="29">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A28)*Contrats!$I$6:$I$13)</f>
@@ -3711,39 +3860,39 @@
       </c>
       <c r="F28" s="29">
         <f>SUMPRODUCT(($A28&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A28-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A28-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="G28" s="29">
         <f>(SUMPRODUCT(($A28&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A28-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A28-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="H28" s="29">
         <f>-($B28*Hypothèses!$B$14+$C28*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I28" s="29">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A28)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A28)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A28)*Contrats!$L$6:$L$13)-IF(AND($B28&gt;0,COUNTIF($B$6:$B28,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J28" s="29">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G28*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B28&gt;0,Hypothèses!$B$40,0)+$G28*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K28" s="29">
         <f>$G28+$E28+$H28+$I28+$J28</f>
-        <v>2339.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L28" s="28">
         <f>L27+$D28+$K28</f>
-        <v>22464.039999999983</v>
+        <v>47006</v>
       </c>
       <c r="M28" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A28&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N28" s="31">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A28&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -3752,11 +3901,11 @@
       </c>
       <c r="B29" s="33">
         <f>$M29+$N29</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C29" s="33">
         <f>IF($B29&lt;=Hypothèses!$B$17,0,IF($M29=0,0,CEILING($M29/Hypothèses!$B$16,1))+IF($N29=0,0,CEILING($N29/Hypothèses!$B$16,1)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D29" s="34">
         <f>SUMPRODUCT((Contrats!$B$6:$B$13=$A29)*Contrats!$I$6:$I$13)</f>
@@ -3768,45 +3917,45 @@
       </c>
       <c r="F29" s="34">
         <f>SUMPRODUCT(($A29&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A29-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A29-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="G29" s="34">
         <f>(SUMPRODUCT(($A29&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$24+Hypothèses!$B$26)*Contrats!$G$6:$G$13)-SUMPRODUCT(($A29-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&gt;=0)*($A29-Hypothèses!$B$26-Contrats!$B$6:$B$13-Hypothèses!$B$24&lt;Hypothèses!$B$29)*Contrats!$K$6:$K$13))*(1-Hypothèses!$B$33)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="H29" s="34">
         <f>-($B29*Hypothèses!$B$14+$C29*Hypothèses!$B$15)</f>
-        <v>-4992.240000000001</v>
+        <v>-3650</v>
       </c>
       <c r="I29" s="34">
-        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A29)*Contrats!$H$6:$H$13)</f>
+        <f>-SUMPRODUCT((Contrats!$B$6:$B$13=$A29)*Contrats!$H$6:$H$13)-SUMPRODUCT((Contrats!$B$6:$B$13=$A29)*Contrats!$L$6:$L$13)-IF(AND($B29&gt;0,COUNTIF($B$6:$B29,"&gt;0")=1),Hypothèses!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J29" s="34">
-        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+$G29*Hypothèses!$B$34)</f>
-        <v>-68</v>
+        <f>-(Hypothèses!$B$19+Hypothèses!$B$20+IF($B29&gt;0,Hypothèses!$B$40,0)+$G29*(Hypothèses!$B$34+Hypothèses!$B$43))</f>
+        <v>-2588</v>
       </c>
       <c r="K29" s="34">
         <f>$G29+$E29+$H29+$I29+$J29</f>
-        <v>2339.7599999999993</v>
+        <v>3762</v>
       </c>
       <c r="L29" s="35">
         <f>L28+$D29+$K29</f>
-        <v>24803.79999999998</v>
+        <v>50768</v>
       </c>
       <c r="M29" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="helpdesk")*($A29&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N29" s="33">
         <f>SUMPRODUCT((Contrats!$C$6:$C$13="support")*($A29&gt;=Contrats!$B$6:$B$13+Hypothèses!$B$23)*Contrats!$D$6:$D$13)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Personnel, onboarding et structure sont négatifs : ce sont des sorties. Le « Résultat » compte les frais d'activation, qui sont acquis, mais pas le dépôt, qui n'est qu'une avance rendue par crédit de facture — le dépôt n'apparaît que dans le cash. Les colonnes M et N (positions par métier) sont masquées : elles servent au calcul du nombre de managers, qui n'est pas mutualisé entre métiers.</t>
+          <t>Personnel, onboarding, équipement, structure et réserves sont négatifs : ce sont des sorties. La structure ne se paie qu'avec du personnel en poste ; le groupe et l'UPS sortent une fois, au premier mois avec du personnel. Le « Résultat » compte les frais d'activation, qui sont acquis, mais pas le dépôt, qui n'est qu'une avance rendue par crédit de facture — le dépôt n'apparaît que dans le cash. Les colonnes M et N (positions par métier) sont masquées : elles servent au calcul du nombre de managers, qui n'est pas mutualisé entre métiers.</t>
         </is>
       </c>
     </row>
@@ -3846,7 +3995,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Tous les contrats actifs, hors onboarding, dépôt, impayés et taxes.</t>
+          <t>Tous les contrats actifs, hors onboarding, équipement, dépôt et impayés.</t>
         </is>
       </c>
     </row>
@@ -3880,29 +4029,29 @@
     <row r="6">
       <c r="A6" s="36" t="str">
         <f>IF(Contrats!$D6="","",IF(Contrats!$A6="",Contrats!$C6,Contrats!$A6))</f>
-        <v>Contrat 1</v>
+        <v>Client A</v>
       </c>
       <c r="B6" s="31">
         <f>IF(Contrats!$D6="","",Contrats!$D6)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" s="29">
         <f>IF(Contrats!$D6="","",Contrats!$G6)</f>
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="D6" s="29">
         <f>IF(Contrats!$D6="","",-Contrats!$D6*Hypothèses!$B$14)</f>
-        <v>-1686.0800000000002</v>
+        <v>-2190</v>
       </c>
       <c r="E6" s="28">
         <f>IF(Contrats!$D6="","",$C6+$D6)</f>
-        <v>2313.92</v>
+        <v>3810</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="36" t="str">
         <f>IF(Contrats!$D7="","",IF(Contrats!$A7="",Contrats!$C7,Contrats!$A7))</f>
-        <v>Contrat 2</v>
+        <v>Client B</v>
       </c>
       <c r="B7" s="31">
         <f>IF(Contrats!$D7="","",Contrats!$D7)</f>
@@ -3910,15 +4059,15 @@
       </c>
       <c r="C7" s="29">
         <f>IF(Contrats!$D7="","",Contrats!$G7)</f>
-        <v>3400</v>
+        <v>4000</v>
       </c>
       <c r="D7" s="29">
         <f>IF(Contrats!$D7="","",-Contrats!$D7*Hypothèses!$B$14)</f>
-        <v>-1686.0800000000002</v>
+        <v>-1460</v>
       </c>
       <c r="E7" s="28">
         <f>IF(Contrats!$D7="","",$C7+$D7)</f>
-        <v>1713.9199999999998</v>
+        <v>2540</v>
       </c>
     </row>
     <row r="8">
@@ -4061,19 +4210,30 @@
       </c>
       <c r="B15" s="38">
         <f>SUM(B6:B13)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15" s="28">
         <f>SUM(C6:C13)</f>
-        <v>7400</v>
+        <v>10000</v>
       </c>
       <c r="D15" s="28">
         <f>SUM(D6:D13)</f>
-        <v>-3372.1600000000003</v>
+        <v>-3650</v>
       </c>
       <c r="E15" s="28">
         <f>SUM(E6:E13)</f>
-        <v>4027.84</v>
+        <v>6350</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Réserves SLA, banque et change</t>
+        </is>
+      </c>
+      <c r="E16" s="29">
+        <f>-C15*(Hypothèses!$B$34+Hypothèses!$B$43)</f>
+        <v>-300.0</v>
       </c>
     </row>
     <row r="17">
@@ -4084,11 +4244,11 @@
       </c>
       <c r="B17" s="31">
         <f>Flux!C29</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E17" s="29">
         <f>-Flux!C29*Hypothèses!$B$15</f>
-        <v>-1620.0800000000002</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="18">
@@ -4102,6 +4262,17 @@
         <v>-68</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Structure du lancement</t>
+        </is>
+      </c>
+      <c r="E19" s="29">
+        <f>-IF(B15&gt;0,Hypothèses!$B$40,0)</f>
+        <v>-2220</v>
+      </c>
+    </row>
     <row r="20">
       <c r="A20" s="39" t="inlineStr">
         <is>
@@ -4109,14 +4280,14 @@
         </is>
       </c>
       <c r="E20" s="40">
-        <f>E15+E17+E18</f>
-        <v>2339.7599999999998</v>
+        <f>E15+E16+E17+E18+E19</f>
+        <v>3762</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>La supervision est comptée globalement, au nombre de managers du dernier mois : elle n'est pas répartie par contrat, parce qu'un manager déclenché par un contrat sert aussi au suivant dans le même métier. C'est le même « résultat mensuel à régime plein » que la page projection-finances-salverys.html et que grille-negociation-salverys.html — CA moins agents, supervision et outils.</t>
+          <t>La supervision est comptée globalement, au nombre de managers du dernier mois : elle n'est pas répartie par contrat, parce qu'un manager déclenché par un contrat sert aussi au suivant dans le même métier. C'est le même « résultat mensuel à régime plein » que la page projection-finances-salverys.html — CA moins réserves, agents, supervision, outils et structure.</t>
         </is>
       </c>
     </row>

</xml_diff>